<commit_message>
feat: separate acrylic parts into dedicated tab in BOM calculator
</commit_message>
<xml_diff>
--- a/Composite_Sheet_Calculator.xlsx
+++ b/Composite_Sheet_Calculator.xlsx
@@ -10,7 +10,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="สรุปภาพรวมทั้งตู้ (Summary)" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ฝั่งนอก (Outer)" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ฝั่งใน (Inner)" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ขนาดแผ่นมาตรฐานและแนวทาง" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="อะคริลิก (Acrylic)" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ขนาดแผ่นมาตรฐานและแนวทาง" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,16 +20,15 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="7">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="#,##0 &quot; ชิ้น&quot;"/>
     <numFmt numFmtId="165" formatCode="#,##0.0000 &quot; m²&quot;"/>
     <numFmt numFmtId="166" formatCode="0 &quot; แผ่น&quot;"/>
-    <numFmt numFmtId="167" formatCode="#,##0.00 &quot; m²&quot;"/>
-    <numFmt numFmtId="168" formatCode="0.0000"/>
-    <numFmt numFmtId="169" formatCode="0.0%"/>
-    <numFmt numFmtId="170" formatCode="#,##0.0000"/>
+    <numFmt numFmtId="167" formatCode="0.0000"/>
+    <numFmt numFmtId="168" formatCode="0.0%"/>
+    <numFmt numFmtId="169" formatCode="#,##0.0000"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="15">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -66,14 +66,20 @@
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
-      <color rgb="001B365D"/>
-      <sz val="10"/>
+      <color rgb="001E8449"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="000E6655"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
       <color rgb="001B365D"/>
-      <sz val="14"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Segoe UI"/>
@@ -84,8 +90,8 @@
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
-      <color rgb="001B365D"/>
-      <sz val="11"/>
+      <color rgb="000E6655"/>
+      <sz val="18"/>
     </font>
     <font>
       <name val="Segoe UI"/>
@@ -112,7 +118,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -133,14 +139,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F4F6F6"/>
-        <bgColor rgb="00F4F6F6"/>
+        <fgColor rgb="00E8F8F5"/>
+        <bgColor rgb="00E8F8F5"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E8F8F5"/>
-        <bgColor rgb="00E8F8F5"/>
+        <fgColor rgb="00D1F2EB"/>
+        <bgColor rgb="00D1F2EB"/>
       </patternFill>
     </fill>
     <fill>
@@ -171,6 +177,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="001B4F72"/>
         <bgColor rgb="001B4F72"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000E6655"/>
+        <bgColor rgb="000E6655"/>
       </patternFill>
     </fill>
   </fills>
@@ -242,7 +254,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -263,34 +275,34 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="4" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="2" fontId="4" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="6" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="7" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="7" fillId="4" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="9" fillId="4" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="8" fillId="5" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="10" fillId="5" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -299,10 +311,10 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -314,19 +326,19 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="170" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="169" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="169" fontId="5" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="168" fontId="5" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -344,7 +356,7 @@
     <xf numFmtId="3" fontId="5" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="169" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="168" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -360,13 +372,13 @@
     <xf numFmtId="0" fontId="2" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="170" fontId="12" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="169" fontId="13" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="169" fontId="4" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="168" fontId="4" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="9" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -382,16 +394,38 @@
     <xf numFmtId="0" fontId="2" fillId="9" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="170" fontId="13" fillId="9" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="169" fontId="14" fillId="9" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="169" fontId="4" fillId="9" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="168" fontId="4" fillId="9" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="4" fillId="5" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="7" fillId="5" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="4" fillId="5" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -760,10 +794,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
@@ -775,21 +809,21 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>📊 สรุปภาพรวมจำนวนแผ่นคอมโพสิตทั้งตู้ (Inner &amp; Outer Combined)</t>
+          <t>📊 สรุปภาพรวมการสั่งซื้อแผ่นคอมโพสิตและอะคริลิก (Bill of Materials)</t>
         </is>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>โครงการ: Narit Vending Machine | เปรียบเทียบและรวมการสั่งซื้อแผ่นคอมโพสิตฝั่งใน (Inner) และฝั่งนอก (Outer)</t>
+          <t>โครงการ: Narit Vending Machine | สรุปแยกตามชนิดวัสดุ: แผ่นคอมโพสิต (ฝั่งใน + ฝั่งนอก) และ แผ่นอะคริลิกใส (Acrylic)</t>
         </is>
       </c>
     </row>
     <row r="4" ht="26" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>หมวดหมู่ / โซน (Section)</t>
+          <t>หมวดหมู่วัสดุ / ส่วนงาน (Material &amp; Section)</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -814,7 +848,7 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>สั่งซื้อแยกฝั่ง (แผ่น)</t>
+          <t>สั่งซื้อ (แผ่น)</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
@@ -826,7 +860,7 @@
     <row r="5" ht="22" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>1. ชิ้นส่วนฝั่งใน (Inner Parts)</t>
+          <t>1. แผ่นคอมโพสิต - ฝั่งใน (Inner Composite)</t>
         </is>
       </c>
       <c r="B5" s="5">
@@ -851,18 +885,18 @@
       </c>
       <c r="G5" s="9" t="inlineStr">
         <is>
-          <t>แผ่นกั้น, ซับในประตู, ฝาครอบหลังใน</t>
+          <t>แผ่นกั้น Partition, กล่องใน, ฝาหลังใน, ซับในประตู</t>
         </is>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>2. ชิ้นส่วนฝั่งนอก (Outer Parts)</t>
+          <t>2. แผ่นคอมโพสิต - ฝั่งนอก (Outer Composite)</t>
         </is>
       </c>
       <c r="B6" s="5">
-        <f>'ฝั่งนอก (Outer)'!D27</f>
+        <f>'ฝั่งนอก (Outer)'!D24</f>
         <v/>
       </c>
       <c r="C6" s="6">
@@ -883,14 +917,14 @@
       </c>
       <c r="G6" s="9" t="inlineStr">
         <is>
-          <t>ฝาบน, ฝาหลัง, ฝาข้างซ้าย-ขวา, ประตูหน้า</t>
+          <t>ฝาบน, ฝาหลัง, ฝาข้างซ้าย-ขวา, บานประตูหน้านอก</t>
         </is>
       </c>
     </row>
     <row r="7" ht="24" customHeight="1">
       <c r="A7" s="10" t="inlineStr">
         <is>
-          <t>รวมแบบสั่งซื้อแยกฝั่ง (Separate Purchasing)</t>
+          <t>⭐ รวมแผ่นคอมโพสิตทั้งตู้ (Total Composite)</t>
         </is>
       </c>
       <c r="B7" s="11">
@@ -910,81 +944,111 @@
         <v/>
       </c>
       <c r="F7" s="14">
-        <f>F5+F6</f>
+        <f>ROUNDUP(D7/'ฝั่งใน (Inner)'!C7, 0)</f>
         <v/>
       </c>
       <c r="G7" s="15" t="inlineStr">
         <is>
-          <t>ผลรวมแผ่นเมื่อปัดเศษแยกแต่ละฝั่ง</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="16" t="inlineStr">
-        <is>
-          <t>💡 แนะนำการสั่งซื้อรวมทั้งตู้
-(Combined Nesting Optimization)
-หากตัดร่วมกันทั้งฝั่งในและฝั่งนอก จะลดเศษเหลือตามมุมได้มากที่สุด</t>
-        </is>
-      </c>
-      <c r="B10" s="17" t="n"/>
-      <c r="C10" s="17" t="n"/>
-      <c r="D10" s="18" t="inlineStr">
-        <is>
-          <t>พื้นที่รวมทั้งตู้ (Gross)</t>
-        </is>
-      </c>
-      <c r="E10" s="17" t="n"/>
-      <c r="F10" s="19" t="inlineStr">
-        <is>
-          <t>จำนวนแผ่นรวมที่ต้องใช้จริง
-(ROUNDUP รวมทั้งตู้)</t>
-        </is>
-      </c>
-      <c r="G10" s="17" t="n"/>
+          <t>คำนวณรวม Nesting ตัดคอมโพสิตทั้งตู้</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="24" customHeight="1">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>3. แผ่นอะคริลิกใส (Acrylic Sheet)</t>
+        </is>
+      </c>
+      <c r="B8" s="5">
+        <f>'อะคริลิก (Acrylic)'!D18</f>
+        <v/>
+      </c>
+      <c r="C8" s="6">
+        <f>'อะคริลิก (Acrylic)'!G6</f>
+        <v/>
+      </c>
+      <c r="D8" s="6">
+        <f>'อะคริลิก (Acrylic)'!G7</f>
+        <v/>
+      </c>
+      <c r="E8" s="7">
+        <f>'อะคริลิก (Acrylic)'!G8</f>
+        <v/>
+      </c>
+      <c r="F8" s="16">
+        <f>'อะคริลิก (Acrylic)'!I6</f>
+        <v/>
+      </c>
+      <c r="G8" s="9" t="inlineStr">
+        <is>
+          <t>ฝาครอบอะคริลิกด้านหน้าและด้านข้าง (แผ่นใส/ตกแต่ง)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="17" t="n"/>
-      <c r="B11" s="17" t="n"/>
-      <c r="C11" s="17" t="n"/>
-      <c r="D11" s="17" t="n"/>
-      <c r="E11" s="17" t="n"/>
-      <c r="F11" s="17" t="n"/>
-      <c r="G11" s="17" t="n"/>
+      <c r="A11" s="17" t="inlineStr">
+        <is>
+          <t>📦 แผ่นอลูมิเนียมคอมโพสิต (Total Composite)
+สั่งซื้อรวมทั้งตู้ (Inner + Outer)</t>
+        </is>
+      </c>
+      <c r="B11" s="18" t="n"/>
+      <c r="C11" s="18" t="n"/>
+      <c r="E11" s="19" t="inlineStr">
+        <is>
+          <t>💎 แผ่นอะคริลิกใส (Acrylic Sheet)
+สำหรับฝาหน้าและฝาข้างขวา</t>
+        </is>
+      </c>
+      <c r="F11" s="18" t="n"/>
+      <c r="G11" s="18" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="17" t="n"/>
-      <c r="B12" s="17" t="n"/>
-      <c r="C12" s="17" t="n"/>
-      <c r="D12" s="20">
-        <f>D7</f>
-        <v/>
-      </c>
-      <c r="E12" s="17" t="n"/>
-      <c r="F12" s="21">
-        <f>ROUNDUP(D7/'ฝั่งใน (Inner)'!C7, 0)</f>
-        <v/>
-      </c>
-      <c r="G12" s="17" t="n"/>
+      <c r="A12" s="18" t="n"/>
+      <c r="B12" s="18" t="n"/>
+      <c r="C12" s="18" t="n"/>
+      <c r="E12" s="18" t="n"/>
+      <c r="F12" s="18" t="n"/>
+      <c r="G12" s="18" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="17" t="n"/>
-      <c r="B13" s="17" t="n"/>
-      <c r="C13" s="17" t="n"/>
-      <c r="D13" s="17" t="n"/>
-      <c r="E13" s="17" t="n"/>
-      <c r="F13" s="17" t="n"/>
-      <c r="G13" s="17" t="n"/>
+      <c r="A13" s="20">
+        <f>F7</f>
+        <v/>
+      </c>
+      <c r="B13" s="18" t="n"/>
+      <c r="C13" s="18" t="n"/>
+      <c r="E13" s="21">
+        <f>F8</f>
+        <v/>
+      </c>
+      <c r="F13" s="18" t="n"/>
+      <c r="G13" s="18" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="18" t="n"/>
+      <c r="B14" s="18" t="n"/>
+      <c r="C14" s="18" t="n"/>
+      <c r="E14" s="18" t="n"/>
+      <c r="F14" s="18" t="n"/>
+      <c r="G14" s="18" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="18" t="n"/>
+      <c r="B15" s="18" t="n"/>
+      <c r="C15" s="18" t="n"/>
+      <c r="E15" s="18" t="n"/>
+      <c r="F15" s="18" t="n"/>
+      <c r="G15" s="18" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="6">
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="F12:G13"/>
-    <mergeCell ref="A10:C13"/>
-    <mergeCell ref="F10:G11"/>
-    <mergeCell ref="D12:E13"/>
+    <mergeCell ref="A11:C12"/>
+    <mergeCell ref="A13:C15"/>
+    <mergeCell ref="E11:G12"/>
+    <mergeCell ref="E13:G15"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="D10:E11"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -996,7 +1060,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J27"/>
+  <dimension ref="A1:J24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1021,14 +1085,14 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="23" t="inlineStr">
         <is>
-          <t>รายการชิ้นส่วนจาก SOLIDWORKS: ฝาบน, ฝาหลัง, ฝาข้าง, ประตู และฝาหน้า</t>
+          <t>รายการชิ้นส่วนจาก SOLIDWORKS: ฝาบน, ฝาหลัง, ฝาข้าง, ประตู และฝาหน้า (เฉพาะแผ่นคอมโพสิต)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="B4" s="24" t="inlineStr">
         <is>
-          <t>⚙️ ข้อมูลแผ่นมาตรฐาน (Standard Sheet Config)</t>
+          <t>⚙️ ข้อมูลแผ่นมาตรฐาน - คอมโพสิต (Standard Sheet Config)</t>
         </is>
       </c>
       <c r="F4" s="24" t="inlineStr">
@@ -1038,11 +1102,11 @@
       </c>
       <c r="I4" s="25" t="inlineStr">
         <is>
-          <t>จำนวนแผ่นที่แนะนำสั่งซื้อ
+          <t>จำนวนแผ่น คอมโพสิต ที่ต้องใช้
 (Recommended to Order)</t>
         </is>
       </c>
-      <c r="J4" s="17" t="n"/>
+      <c r="J4" s="18" t="n"/>
     </row>
     <row r="5">
       <c r="B5" s="26" t="inlineStr">
@@ -1064,7 +1128,7 @@
         </is>
       </c>
       <c r="G5" s="30">
-        <f>SUM(D12:D26)</f>
+        <f>SUM(D12:D23)</f>
         <v/>
       </c>
       <c r="H5" s="28" t="inlineStr">
@@ -1072,8 +1136,8 @@
           <t>ชิ้น (pcs)</t>
         </is>
       </c>
-      <c r="I5" s="17" t="n"/>
-      <c r="J5" s="17" t="n"/>
+      <c r="I5" s="18" t="n"/>
+      <c r="J5" s="18" t="n"/>
     </row>
     <row r="6">
       <c r="B6" s="26" t="inlineStr">
@@ -1095,7 +1159,7 @@
         </is>
       </c>
       <c r="G6" s="31">
-        <f>SUM(G12:G26)</f>
+        <f>SUM(G12:G23)</f>
         <v/>
       </c>
       <c r="H6" s="28" t="inlineStr">
@@ -1103,11 +1167,11 @@
           <t>ตร.ม. (m²)</t>
         </is>
       </c>
-      <c r="I6" s="21">
+      <c r="I6" s="20">
         <f>ROUNDUP(G8, 0)</f>
         <v/>
       </c>
-      <c r="J6" s="17" t="n"/>
+      <c r="J6" s="18" t="n"/>
     </row>
     <row r="7">
       <c r="B7" s="26" t="inlineStr">
@@ -1138,8 +1202,8 @@
           <t>ตร.ม. (m²)</t>
         </is>
       </c>
-      <c r="I7" s="17" t="n"/>
-      <c r="J7" s="17" t="n"/>
+      <c r="I7" s="18" t="n"/>
+      <c r="J7" s="18" t="n"/>
     </row>
     <row r="8">
       <c r="B8" s="26" t="inlineStr">
@@ -1169,8 +1233,8 @@
           <t>แผ่น (sheets)</t>
         </is>
       </c>
-      <c r="I8" s="17" t="n"/>
-      <c r="J8" s="17" t="n"/>
+      <c r="I8" s="18" t="n"/>
+      <c r="J8" s="18" t="n"/>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="35" t="inlineStr">
@@ -1223,8 +1287,8 @@
       </c>
       <c r="I11" s="35" t="inlineStr">
         <is>
-          <t>หมายเหตุการตัด / พับ
-Remarks &amp; Bending Note</t>
+          <t>หมายเหตุการตัด / พับ / ติดตั้ง
+Remarks &amp; Notes</t>
         </is>
       </c>
     </row>
@@ -1432,12 +1496,12 @@
       </c>
       <c r="B18" s="37" t="inlineStr">
         <is>
-          <t>Arcylic Cover Front 2-st</t>
+          <t>Cover Front 2-Bending-st</t>
         </is>
       </c>
       <c r="C18" s="26" t="inlineStr">
         <is>
-          <t>ฝาครอบหน้า 2 (อะคริลิก/คอมโพสิต)</t>
+          <t>ฝาครอบหน้า 2 (พับขึ้นรูป)</t>
         </is>
       </c>
       <c r="D18" s="38" t="n">
@@ -1455,7 +1519,7 @@
       </c>
       <c r="I18" s="28" t="inlineStr">
         <is>
-          <t>เช็คสเปกว่าใช้ อะคริลิก หรือ คอมโพสิต</t>
+          <t>ชิ้นงานพับขอบ Bending</t>
         </is>
       </c>
     </row>
@@ -1465,12 +1529,12 @@
       </c>
       <c r="B19" s="37" t="inlineStr">
         <is>
-          <t>Arcylic Cover Front-st</t>
+          <t>Cover Right Side 1-Bending-st</t>
         </is>
       </c>
       <c r="C19" s="26" t="inlineStr">
         <is>
-          <t>ฝาครอบหน้า (อะคริลิก/คอมโพสิต)</t>
+          <t>ฝาครอบข้างขวา 1 (พับขึ้นรูป)</t>
         </is>
       </c>
       <c r="D19" s="38" t="n">
@@ -1488,7 +1552,7 @@
       </c>
       <c r="I19" s="28" t="inlineStr">
         <is>
-          <t>เช็คสเปกว่าใช้ อะคริลิก หรือ คอมโพสิต</t>
+          <t>ชิ้นงานพับขอบ Bending</t>
         </is>
       </c>
     </row>
@@ -1498,12 +1562,12 @@
       </c>
       <c r="B20" s="37" t="inlineStr">
         <is>
-          <t>Cover Front 2-Bending-st</t>
+          <t>Cover Right Side 2-Bending-st</t>
         </is>
       </c>
       <c r="C20" s="26" t="inlineStr">
         <is>
-          <t>ฝาครอบหน้า 2 (พับขึ้นรูป)</t>
+          <t>ฝาครอบข้างขวา 2 (พับขึ้นรูป)</t>
         </is>
       </c>
       <c r="D20" s="38" t="n">
@@ -1525,22 +1589,22 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="21" customHeight="1">
-      <c r="A21" s="36" t="n">
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="40" t="n">
         <v>10</v>
       </c>
-      <c r="B21" s="37" t="inlineStr">
-        <is>
-          <t>Arcylic Cover Right -side-st</t>
-        </is>
-      </c>
-      <c r="C21" s="26" t="inlineStr">
-        <is>
-          <t>ฝาครอบข้างขวา (อะคริลิก/คอมโพสิต)</t>
+      <c r="B21" s="28" t="inlineStr">
+        <is>
+          <t>สำรองชิ้นส่วนเพิ่มเติม 1 (Extra Part)</t>
+        </is>
+      </c>
+      <c r="C21" s="28" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="D21" s="38" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E21" s="27" t="inlineStr"/>
       <c r="F21" s="27" t="inlineStr"/>
@@ -1552,28 +1616,24 @@
         <f>IF($C$7&gt;0, G21/$C$7, 0)</f>
         <v/>
       </c>
-      <c r="I21" s="28" t="inlineStr">
-        <is>
-          <t>เช็คสเปกว่าใช้ อะคริลิก หรือ คอมโพสิต</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="21" customHeight="1">
-      <c r="A22" s="36" t="n">
+      <c r="I21" s="28" t="inlineStr"/>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="40" t="n">
         <v>11</v>
       </c>
-      <c r="B22" s="37" t="inlineStr">
-        <is>
-          <t>Cover Right Side 1-Bending-st</t>
-        </is>
-      </c>
-      <c r="C22" s="26" t="inlineStr">
-        <is>
-          <t>ฝาครอบข้างขวา 1 (พับขึ้นรูป)</t>
+      <c r="B22" s="28" t="inlineStr">
+        <is>
+          <t>สำรองชิ้นส่วนเพิ่มเติม 2 (Extra Part)</t>
+        </is>
+      </c>
+      <c r="C22" s="28" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="D22" s="38" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E22" s="27" t="inlineStr"/>
       <c r="F22" s="27" t="inlineStr"/>
@@ -1585,28 +1645,24 @@
         <f>IF($C$7&gt;0, G22/$C$7, 0)</f>
         <v/>
       </c>
-      <c r="I22" s="28" t="inlineStr">
-        <is>
-          <t>ชิ้นงานพับขอบ Bending</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="21" customHeight="1">
-      <c r="A23" s="36" t="n">
+      <c r="I22" s="28" t="inlineStr"/>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="40" t="n">
         <v>12</v>
       </c>
-      <c r="B23" s="37" t="inlineStr">
-        <is>
-          <t>Cover Right Side 2-Bending-st</t>
-        </is>
-      </c>
-      <c r="C23" s="26" t="inlineStr">
-        <is>
-          <t>ฝาครอบข้างขวา 2 (พับขึ้นรูป)</t>
+      <c r="B23" s="28" t="inlineStr">
+        <is>
+          <t>สำรองชิ้นส่วนเพิ่มเติม 3 (Extra Part)</t>
+        </is>
+      </c>
+      <c r="C23" s="28" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="D23" s="38" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E23" s="27" t="inlineStr"/>
       <c r="F23" s="27" t="inlineStr"/>
@@ -1618,140 +1674,49 @@
         <f>IF($C$7&gt;0, G23/$C$7, 0)</f>
         <v/>
       </c>
-      <c r="I23" s="28" t="inlineStr">
-        <is>
-          <t>ชิ้นงานพับขอบ Bending</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="20" customHeight="1">
-      <c r="A24" s="40" t="n">
-        <v>13</v>
-      </c>
-      <c r="B24" s="28" t="inlineStr">
-        <is>
-          <t>สำรองชิ้นส่วนเพิ่มเติม 1 (Extra Part)</t>
-        </is>
-      </c>
-      <c r="C24" s="28" t="inlineStr">
+      <c r="I23" s="28" t="inlineStr"/>
+    </row>
+    <row r="24" ht="24" customHeight="1">
+      <c r="A24" s="41" t="inlineStr">
+        <is>
+          <t>รวมทั้งหมด (Sub-Total)</t>
+        </is>
+      </c>
+      <c r="B24" s="42" t="n"/>
+      <c r="C24" s="42" t="n"/>
+      <c r="D24" s="43">
+        <f>SUM(D12:D23)</f>
+        <v/>
+      </c>
+      <c r="E24" s="44" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="D24" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="E24" s="27" t="inlineStr"/>
-      <c r="F24" s="27" t="inlineStr"/>
-      <c r="G24" s="31">
-        <f>IF(AND(ISNUMBER(E24),ISNUMBER(F24),E24&gt;0,F24&gt;0), D24*(E24*F24)/1000000, 0)</f>
-        <v/>
-      </c>
-      <c r="H24" s="39">
-        <f>IF($C$7&gt;0, G24/$C$7, 0)</f>
-        <v/>
-      </c>
-      <c r="I24" s="28" t="inlineStr"/>
-    </row>
-    <row r="25" ht="20" customHeight="1">
-      <c r="A25" s="40" t="n">
-        <v>14</v>
-      </c>
-      <c r="B25" s="28" t="inlineStr">
-        <is>
-          <t>สำรองชิ้นส่วนเพิ่มเติม 2 (Extra Part)</t>
-        </is>
-      </c>
-      <c r="C25" s="28" t="inlineStr">
+      <c r="F24" s="44" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="D25" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="E25" s="27" t="inlineStr"/>
-      <c r="F25" s="27" t="inlineStr"/>
-      <c r="G25" s="31">
-        <f>IF(AND(ISNUMBER(E25),ISNUMBER(F25),E25&gt;0,F25&gt;0), D25*(E25*F25)/1000000, 0)</f>
-        <v/>
-      </c>
-      <c r="H25" s="39">
-        <f>IF($C$7&gt;0, G25/$C$7, 0)</f>
-        <v/>
-      </c>
-      <c r="I25" s="28" t="inlineStr"/>
-    </row>
-    <row r="26" ht="20" customHeight="1">
-      <c r="A26" s="40" t="n">
-        <v>15</v>
-      </c>
-      <c r="B26" s="28" t="inlineStr">
-        <is>
-          <t>สำรองชิ้นส่วนเพิ่มเติม 3 (Extra Part)</t>
-        </is>
-      </c>
-      <c r="C26" s="28" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D26" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="E26" s="27" t="inlineStr"/>
-      <c r="F26" s="27" t="inlineStr"/>
-      <c r="G26" s="31">
-        <f>IF(AND(ISNUMBER(E26),ISNUMBER(F26),E26&gt;0,F26&gt;0), D26*(E26*F26)/1000000, 0)</f>
-        <v/>
-      </c>
-      <c r="H26" s="39">
-        <f>IF($C$7&gt;0, G26/$C$7, 0)</f>
-        <v/>
-      </c>
-      <c r="I26" s="28" t="inlineStr"/>
-    </row>
-    <row r="27" ht="24" customHeight="1">
-      <c r="A27" s="41" t="inlineStr">
-        <is>
-          <t>รวมทั้งหมด (Sub-Total)</t>
-        </is>
-      </c>
-      <c r="B27" s="42" t="n"/>
-      <c r="C27" s="42" t="n"/>
-      <c r="D27" s="43">
-        <f>SUM(D12:D26)</f>
-        <v/>
-      </c>
-      <c r="E27" s="44" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F27" s="44" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G27" s="45">
-        <f>SUM(G12:G26)</f>
-        <v/>
-      </c>
-      <c r="H27" s="46">
-        <f>SUM(H12:H26)</f>
-        <v/>
-      </c>
-      <c r="I27" s="42" t="inlineStr"/>
+      <c r="G24" s="45">
+        <f>SUM(G12:G23)</f>
+        <v/>
+      </c>
+      <c r="H24" s="46">
+        <f>SUM(H12:H23)</f>
+        <v/>
+      </c>
+      <c r="I24" s="42" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="I4:J5"/>
     <mergeCell ref="B4:D4"/>
-    <mergeCell ref="A27:C27"/>
     <mergeCell ref="F4:H4"/>
     <mergeCell ref="A2:J2"/>
     <mergeCell ref="I6:J8"/>
+    <mergeCell ref="A24:C24"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1795,7 +1760,7 @@
     <row r="4">
       <c r="B4" s="24" t="inlineStr">
         <is>
-          <t>⚙️ ข้อมูลแผ่นมาตรฐาน (Standard Sheet Config)</t>
+          <t>⚙️ ข้อมูลแผ่นมาตรฐาน - คอมโพสิต (Standard Sheet Config)</t>
         </is>
       </c>
       <c r="F4" s="24" t="inlineStr">
@@ -1805,11 +1770,11 @@
       </c>
       <c r="I4" s="47" t="inlineStr">
         <is>
-          <t>จำนวนแผ่นที่แนะนำสั่งซื้อ
+          <t>จำนวนแผ่น คอมโพสิต ที่ต้องใช้
 (Recommended to Order)</t>
         </is>
       </c>
-      <c r="J4" s="17" t="n"/>
+      <c r="J4" s="18" t="n"/>
     </row>
     <row r="5">
       <c r="B5" s="26" t="inlineStr">
@@ -1839,8 +1804,8 @@
           <t>ชิ้น (pcs)</t>
         </is>
       </c>
-      <c r="I5" s="17" t="n"/>
-      <c r="J5" s="17" t="n"/>
+      <c r="I5" s="18" t="n"/>
+      <c r="J5" s="18" t="n"/>
     </row>
     <row r="6">
       <c r="B6" s="26" t="inlineStr">
@@ -1870,11 +1835,11 @@
           <t>ตร.ม. (m²)</t>
         </is>
       </c>
-      <c r="I6" s="21">
+      <c r="I6" s="20">
         <f>ROUNDUP(G8, 0)</f>
         <v/>
       </c>
-      <c r="J6" s="17" t="n"/>
+      <c r="J6" s="18" t="n"/>
     </row>
     <row r="7">
       <c r="B7" s="26" t="inlineStr">
@@ -1905,8 +1870,8 @@
           <t>ตร.ม. (m²)</t>
         </is>
       </c>
-      <c r="I7" s="17" t="n"/>
-      <c r="J7" s="17" t="n"/>
+      <c r="I7" s="18" t="n"/>
+      <c r="J7" s="18" t="n"/>
     </row>
     <row r="8">
       <c r="B8" s="26" t="inlineStr">
@@ -1936,8 +1901,8 @@
           <t>แผ่น (sheets)</t>
         </is>
       </c>
-      <c r="I8" s="17" t="n"/>
-      <c r="J8" s="17" t="n"/>
+      <c r="I8" s="18" t="n"/>
+      <c r="J8" s="18" t="n"/>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="48" t="inlineStr">
@@ -1990,8 +1955,8 @@
       </c>
       <c r="I11" s="48" t="inlineStr">
         <is>
-          <t>หมายเหตุการตัด / พับ
-Remarks &amp; Bending Note</t>
+          <t>หมายเหตุการตัด / พับ / ติดตั้ง
+Remarks &amp; Notes</t>
         </is>
       </c>
     </row>
@@ -2431,7 +2396,477 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:J18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="22" t="inlineStr">
+        <is>
+          <t>ตารางคำนวณแผ่นอะคริลิก (Acrylic Sheet Requirement)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="23" t="inlineStr">
+        <is>
+          <t>รายการชิ้นส่วนอะคริลิกจาก SOLIDWORKS: ฝาครอบด้านหน้าและฝาครอบด้านข้าง</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="24" t="inlineStr">
+        <is>
+          <t>⚙️ ข้อมูลแผ่นมาตรฐาน - อะคริลิก (Standard Sheet Config)</t>
+        </is>
+      </c>
+      <c r="F4" s="24" t="inlineStr">
+        <is>
+          <t>📊 ผลลัพธ์การคำนวณ (Calculation Summary)</t>
+        </is>
+      </c>
+      <c r="I4" s="55" t="inlineStr">
+        <is>
+          <t>จำนวนแผ่น อะคริลิก ที่ต้องใช้
+(Recommended to Order)</t>
+        </is>
+      </c>
+      <c r="J4" s="18" t="n"/>
+    </row>
+    <row r="5">
+      <c r="B5" s="26" t="inlineStr">
+        <is>
+          <t>ความกว้างแผ่นมาตรฐาน (Sheet Width)</t>
+        </is>
+      </c>
+      <c r="C5" s="27" t="n">
+        <v>1220</v>
+      </c>
+      <c r="D5" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> มม. (mm)</t>
+        </is>
+      </c>
+      <c r="F5" s="29" t="inlineStr">
+        <is>
+          <t>จำนวนชิ้นงานทั้งหมด (Total Quantity)</t>
+        </is>
+      </c>
+      <c r="G5" s="30">
+        <f>SUM(D12:D17)</f>
+        <v/>
+      </c>
+      <c r="H5" s="28" t="inlineStr">
+        <is>
+          <t>ชิ้น (pcs)</t>
+        </is>
+      </c>
+      <c r="I5" s="18" t="n"/>
+      <c r="J5" s="18" t="n"/>
+    </row>
+    <row r="6">
+      <c r="B6" s="26" t="inlineStr">
+        <is>
+          <t>ความยาวแผ่นมาตรฐาน (Sheet Length)</t>
+        </is>
+      </c>
+      <c r="C6" s="27" t="n">
+        <v>2440</v>
+      </c>
+      <c r="D6" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> มม. (mm)</t>
+        </is>
+      </c>
+      <c r="F6" s="29" t="inlineStr">
+        <is>
+          <t>พื้นที่ชิ้นงานสุทธิ (Net Total Area)</t>
+        </is>
+      </c>
+      <c r="G6" s="31">
+        <f>SUM(G12:G17)</f>
+        <v/>
+      </c>
+      <c r="H6" s="28" t="inlineStr">
+        <is>
+          <t>ตร.ม. (m²)</t>
+        </is>
+      </c>
+      <c r="I6" s="20">
+        <f>ROUNDUP(G8, 0)</f>
+        <v/>
+      </c>
+      <c r="J6" s="18" t="n"/>
+    </row>
+    <row r="7">
+      <c r="B7" s="26" t="inlineStr">
+        <is>
+          <t>พื้นที่ต่อ 1 แผ่นมาตรฐาน (Area/Sheet)</t>
+        </is>
+      </c>
+      <c r="C7" s="32">
+        <f>(C5*C6)/1000000</f>
+        <v/>
+      </c>
+      <c r="D7" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> ตร.ม. (m²)</t>
+        </is>
+      </c>
+      <c r="F7" s="29" t="inlineStr">
+        <is>
+          <t>พื้นที่รวมเผื่อเศษตัด (Gross Area with Waste)</t>
+        </is>
+      </c>
+      <c r="G7" s="31">
+        <f>G6*(1+C8)</f>
+        <v/>
+      </c>
+      <c r="H7" s="28" t="inlineStr">
+        <is>
+          <t>ตร.ม. (m²)</t>
+        </is>
+      </c>
+      <c r="I7" s="18" t="n"/>
+      <c r="J7" s="18" t="n"/>
+    </row>
+    <row r="8">
+      <c r="B8" s="26" t="inlineStr">
+        <is>
+          <t>เผื่อเศษตัด/พับ/โครงสร้าง (Waste Factor)</t>
+        </is>
+      </c>
+      <c r="C8" s="33" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="D8" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> (15%)</t>
+        </is>
+      </c>
+      <c r="F8" s="29" t="inlineStr">
+        <is>
+          <t>จำนวนแผ่นตามทฤษฎี (Theoretical Sheets)</t>
+        </is>
+      </c>
+      <c r="G8" s="34">
+        <f>G7/C7</f>
+        <v/>
+      </c>
+      <c r="H8" s="28" t="inlineStr">
+        <is>
+          <t>แผ่น (sheets)</t>
+        </is>
+      </c>
+      <c r="I8" s="18" t="n"/>
+      <c r="J8" s="18" t="n"/>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="56" t="inlineStr">
+        <is>
+          <t>ลำดับ
+No.</t>
+        </is>
+      </c>
+      <c r="B11" s="56" t="inlineStr">
+        <is>
+          <t>รหัส / ชื่อชิ้นงาน (SOLIDWORKS)
+Part Name</t>
+        </is>
+      </c>
+      <c r="C11" s="56" t="inlineStr">
+        <is>
+          <t>ลักษณะชิ้นงาน / ตำแหน่ง
+Description</t>
+        </is>
+      </c>
+      <c r="D11" s="56" t="inlineStr">
+        <is>
+          <t>จำนวน
+Qty (pcs)</t>
+        </is>
+      </c>
+      <c r="E11" s="56" t="inlineStr">
+        <is>
+          <t>กว้างคลี่ (W)
+Width (mm)</t>
+        </is>
+      </c>
+      <c r="F11" s="56" t="inlineStr">
+        <is>
+          <t>ยาวคลี่ (L)
+Length (mm)</t>
+        </is>
+      </c>
+      <c r="G11" s="56" t="inlineStr">
+        <is>
+          <t>พื้นที่รวม
+Total Area (m²)</t>
+        </is>
+      </c>
+      <c r="H11" s="56" t="inlineStr">
+        <is>
+          <t>สัดส่วนต่อแผ่น
+% of Sheet</t>
+        </is>
+      </c>
+      <c r="I11" s="56" t="inlineStr">
+        <is>
+          <t>หมายเหตุการตัด / พับ / ติดตั้ง
+Remarks &amp; Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="21" customHeight="1">
+      <c r="A12" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="B12" s="37" t="inlineStr">
+        <is>
+          <t>Arcylic Cover Front 2-st</t>
+        </is>
+      </c>
+      <c r="C12" s="26" t="inlineStr">
+        <is>
+          <t>ฝาครอบหน้า 2 (แผ่นอะคริลิกใส/ป้ายไฟ)</t>
+        </is>
+      </c>
+      <c r="D12" s="38" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" s="27" t="inlineStr"/>
+      <c r="F12" s="27" t="inlineStr"/>
+      <c r="G12" s="31">
+        <f>IF(AND(ISNUMBER(E12),ISNUMBER(F12),E12&gt;0,F12&gt;0), D12*(E12*F12)/1000000, 0)</f>
+        <v/>
+      </c>
+      <c r="H12" s="39">
+        <f>IF($C$7&gt;0, G12/$C$7, 0)</f>
+        <v/>
+      </c>
+      <c r="I12" s="28" t="inlineStr">
+        <is>
+          <t>ตัดเลเซอร์ Laser Cut / ขัดขอบ</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="21" customHeight="1">
+      <c r="A13" s="36" t="n">
+        <v>2</v>
+      </c>
+      <c r="B13" s="37" t="inlineStr">
+        <is>
+          <t>Arcylic Cover Front-st</t>
+        </is>
+      </c>
+      <c r="C13" s="26" t="inlineStr">
+        <is>
+          <t>ฝาครอบหน้า (แผ่นอะคริลิกใส/ช่องมอง)</t>
+        </is>
+      </c>
+      <c r="D13" s="38" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" s="27" t="inlineStr"/>
+      <c r="F13" s="27" t="inlineStr"/>
+      <c r="G13" s="31">
+        <f>IF(AND(ISNUMBER(E13),ISNUMBER(F13),E13&gt;0,F13&gt;0), D13*(E13*F13)/1000000, 0)</f>
+        <v/>
+      </c>
+      <c r="H13" s="39">
+        <f>IF($C$7&gt;0, G13/$C$7, 0)</f>
+        <v/>
+      </c>
+      <c r="I13" s="28" t="inlineStr">
+        <is>
+          <t>ตัดเลเซอร์ Laser Cut / ขัดขอบ</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="21" customHeight="1">
+      <c r="A14" s="36" t="n">
+        <v>3</v>
+      </c>
+      <c r="B14" s="37" t="inlineStr">
+        <is>
+          <t>Arcylic Cover Right -side-st</t>
+        </is>
+      </c>
+      <c r="C14" s="26" t="inlineStr">
+        <is>
+          <t>ฝาครอบข้างขวา (แผ่นอะคริลิกใส/แสดงผล)</t>
+        </is>
+      </c>
+      <c r="D14" s="38" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" s="27" t="inlineStr"/>
+      <c r="F14" s="27" t="inlineStr"/>
+      <c r="G14" s="31">
+        <f>IF(AND(ISNUMBER(E14),ISNUMBER(F14),E14&gt;0,F14&gt;0), D14*(E14*F14)/1000000, 0)</f>
+        <v/>
+      </c>
+      <c r="H14" s="39">
+        <f>IF($C$7&gt;0, G14/$C$7, 0)</f>
+        <v/>
+      </c>
+      <c r="I14" s="28" t="inlineStr">
+        <is>
+          <t>ตัดเลเซอร์ Laser Cut / ขัดขอบ</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="40" t="n">
+        <v>4</v>
+      </c>
+      <c r="B15" s="28" t="inlineStr">
+        <is>
+          <t>สำรองชิ้นส่วนเพิ่มเติม 1 (Extra Part)</t>
+        </is>
+      </c>
+      <c r="C15" s="28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D15" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" s="27" t="inlineStr"/>
+      <c r="F15" s="27" t="inlineStr"/>
+      <c r="G15" s="31">
+        <f>IF(AND(ISNUMBER(E15),ISNUMBER(F15),E15&gt;0,F15&gt;0), D15*(E15*F15)/1000000, 0)</f>
+        <v/>
+      </c>
+      <c r="H15" s="39">
+        <f>IF($C$7&gt;0, G15/$C$7, 0)</f>
+        <v/>
+      </c>
+      <c r="I15" s="28" t="inlineStr"/>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="40" t="n">
+        <v>5</v>
+      </c>
+      <c r="B16" s="28" t="inlineStr">
+        <is>
+          <t>สำรองชิ้นส่วนเพิ่มเติม 2 (Extra Part)</t>
+        </is>
+      </c>
+      <c r="C16" s="28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D16" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" s="27" t="inlineStr"/>
+      <c r="F16" s="27" t="inlineStr"/>
+      <c r="G16" s="31">
+        <f>IF(AND(ISNUMBER(E16),ISNUMBER(F16),E16&gt;0,F16&gt;0), D16*(E16*F16)/1000000, 0)</f>
+        <v/>
+      </c>
+      <c r="H16" s="39">
+        <f>IF($C$7&gt;0, G16/$C$7, 0)</f>
+        <v/>
+      </c>
+      <c r="I16" s="28" t="inlineStr"/>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="40" t="n">
+        <v>6</v>
+      </c>
+      <c r="B17" s="28" t="inlineStr">
+        <is>
+          <t>สำรองชิ้นส่วนเพิ่มเติม 3 (Extra Part)</t>
+        </is>
+      </c>
+      <c r="C17" s="28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D17" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" s="27" t="inlineStr"/>
+      <c r="F17" s="27" t="inlineStr"/>
+      <c r="G17" s="31">
+        <f>IF(AND(ISNUMBER(E17),ISNUMBER(F17),E17&gt;0,F17&gt;0), D17*(E17*F17)/1000000, 0)</f>
+        <v/>
+      </c>
+      <c r="H17" s="39">
+        <f>IF($C$7&gt;0, G17/$C$7, 0)</f>
+        <v/>
+      </c>
+      <c r="I17" s="28" t="inlineStr"/>
+    </row>
+    <row r="18" ht="24" customHeight="1">
+      <c r="A18" s="57" t="inlineStr">
+        <is>
+          <t>รวมทั้งหมด (Sub-Total)</t>
+        </is>
+      </c>
+      <c r="B18" s="58" t="n"/>
+      <c r="C18" s="58" t="n"/>
+      <c r="D18" s="59">
+        <f>SUM(D12:D17)</f>
+        <v/>
+      </c>
+      <c r="E18" s="60" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F18" s="60" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G18" s="61">
+        <f>SUM(G12:G17)</f>
+        <v/>
+      </c>
+      <c r="H18" s="62">
+        <f>SUM(H12:H17)</f>
+        <v/>
+      </c>
+      <c r="I18" s="58" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="I4:J5"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="A18:C18"/>
+    <mergeCell ref="F4:H4"/>
+    <mergeCell ref="A2:J2"/>
+    <mergeCell ref="I6:J8"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -2445,80 +2880,60 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>ข้อมูลอ้างอิงขนาดแผ่นอลูมิเนียมคอมโพสิต (Aluminum Composite Sheet Standards)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="25" customHeight="1">
-      <c r="A3" s="3" t="inlineStr">
+          <t>ข้อมูลอ้างอิงขนาดแผ่นอลูมิเนียมคอมโพสิตและแผ่นอะคริลิก</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="63" t="inlineStr">
+        <is>
+          <t>1. ขนาดแผ่นอลูมิเนียมคอมโพสิตมาตรฐาน (Aluminum Composite Standard Sizes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="25" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>ขนาดมาตรฐาน (Standard Size)</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>กว้าง (W) มม.</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>ยาว (L) มม.</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>พื้นที่ (ตร.ม./แผ่น)</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>ความหนารวมทั่วไป</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>การใช้งานที่นิยม</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="37" t="inlineStr">
-        <is>
-          <t>4 x 8 ฟุต (มาตรฐานสากล - นิยมที่สุด)</t>
-        </is>
-      </c>
-      <c r="B4" s="55" t="n">
-        <v>1220</v>
-      </c>
-      <c r="C4" s="55" t="n">
-        <v>2440</v>
-      </c>
-      <c r="D4" s="32">
-        <f>B4*C4/1000000</f>
-        <v/>
-      </c>
-      <c r="E4" s="26" t="inlineStr">
-        <is>
-          <t>3 มม. / 4 มม.</t>
-        </is>
-      </c>
-      <c r="F4" s="26" t="inlineStr">
-        <is>
-          <t>โครงสร้างตู้, พาร์ทิชัน, ป้าย</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="37" t="inlineStr">
         <is>
-          <t>1.25 x 2.50 เมตร (ไซส์ยุโรป)</t>
-        </is>
-      </c>
-      <c r="B5" s="55" t="n">
-        <v>1250</v>
-      </c>
-      <c r="C5" s="55" t="n">
-        <v>2500</v>
+          <t>4 x 8 ฟุต (มาตรฐานสากล - นิยมที่สุด)</t>
+        </is>
+      </c>
+      <c r="B5" s="64" t="n">
+        <v>1220</v>
+      </c>
+      <c r="C5" s="64" t="n">
+        <v>2440</v>
       </c>
       <c r="D5" s="32">
         <f>B5*C5/1000000</f>
@@ -2526,26 +2941,26 @@
       </c>
       <c r="E5" s="26" t="inlineStr">
         <is>
-          <t>4 มม.</t>
+          <t>3 มม. / 4 มม.</t>
         </is>
       </c>
       <c r="F5" s="26" t="inlineStr">
         <is>
-          <t>งานอาคาร, ผนังตู้ขนาดใหญ่</t>
+          <t>โครงสร้างตู้, พาร์ทิชัน, ฝาครอบ</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="37" t="inlineStr">
         <is>
-          <t>4 x 10 ฟุต (แผ่นยาว)</t>
-        </is>
-      </c>
-      <c r="B6" s="55" t="n">
-        <v>1220</v>
-      </c>
-      <c r="C6" s="55" t="n">
-        <v>3050</v>
+          <t>1.25 x 2.50 เมตร (ไซส์ยุโรป)</t>
+        </is>
+      </c>
+      <c r="B6" s="64" t="n">
+        <v>1250</v>
+      </c>
+      <c r="C6" s="64" t="n">
+        <v>2500</v>
       </c>
       <c r="D6" s="32">
         <f>B6*C6/1000000</f>
@@ -2558,21 +2973,21 @@
       </c>
       <c r="F6" s="26" t="inlineStr">
         <is>
-          <t>ฝาหลังตู้สูง, ชิ้นส่วนยาวต่อเนื่อง</t>
+          <t>งานอาคาร, ผนังตู้ขนาดใหญ่</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="37" t="inlineStr">
         <is>
-          <t>5 x 10 ฟุต (แผ่นหน้ากว้าง)</t>
-        </is>
-      </c>
-      <c r="B7" s="55" t="n">
-        <v>1500</v>
-      </c>
-      <c r="C7" s="55" t="n">
-        <v>3000</v>
+          <t>4 x 10 ฟุต (แผ่นยาว)</t>
+        </is>
+      </c>
+      <c r="B7" s="64" t="n">
+        <v>1220</v>
+      </c>
+      <c r="C7" s="64" t="n">
+        <v>3050</v>
       </c>
       <c r="D7" s="32">
         <f>B7*C7/1000000</f>
@@ -2585,69 +3000,229 @@
       </c>
       <c r="F7" s="26" t="inlineStr">
         <is>
+          <t>ฝาหลังตู้สูง, ชิ้นส่วนยาวต่อเนื่อง</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="37" t="inlineStr">
+        <is>
+          <t>5 x 10 ฟุต (แผ่นหน้ากว้าง)</t>
+        </is>
+      </c>
+      <c r="B8" s="64" t="n">
+        <v>1500</v>
+      </c>
+      <c r="C8" s="64" t="n">
+        <v>3000</v>
+      </c>
+      <c r="D8" s="32">
+        <f>B8*C8/1000000</f>
+        <v/>
+      </c>
+      <c r="E8" s="26" t="inlineStr">
+        <is>
+          <t>4 มม.</t>
+        </is>
+      </c>
+      <c r="F8" s="26" t="inlineStr">
+        <is>
           <t>ชิ้นงานขนาดใหญ่ลดรอยต่อ</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="56" t="inlineStr">
-        <is>
-          <t>📐 เทคนิคการคำนวณขนาดคลี่สำหรับงานพับแผ่นคอมโพสิต (V-Groove Bending Allowance)</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="57" t="inlineStr">
-        <is>
-          <t>1. การพับแผ่นอลูมิเนียมคอมโพสิต นิยมใช้ใบเซาะร่อง V-Groove 90° หรือ 135° ด้านหลัง โดยเหลือชั้นแกนพลาสติกและอลูมิเนียมผิวหน้าไว้ประมาณ 0.5 - 0.8 มม.</t>
+      <c r="A10" s="63" t="inlineStr">
+        <is>
+          <t>2. ขนาดแผ่นอะคริลิกมาตรฐาน (Acrylic Sheet Standard Sizes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="25" customHeight="1">
+      <c r="A11" s="56" t="inlineStr">
+        <is>
+          <t>ขนาดแผ่นอะคริลิก</t>
+        </is>
+      </c>
+      <c r="B11" s="56" t="inlineStr">
+        <is>
+          <t>กว้าง (W) มม.</t>
+        </is>
+      </c>
+      <c r="C11" s="56" t="inlineStr">
+        <is>
+          <t>ยาว (L) มม.</t>
+        </is>
+      </c>
+      <c r="D11" s="56" t="inlineStr">
+        <is>
+          <t>พื้นที่ (ตร.ม./แผ่น)</t>
+        </is>
+      </c>
+      <c r="E11" s="56" t="inlineStr">
+        <is>
+          <t>ความหนาทั่วไป</t>
+        </is>
+      </c>
+      <c r="F11" s="56" t="inlineStr">
+        <is>
+          <t>คุณสมบัติ/การใช้งาน</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="57" t="inlineStr">
-        <is>
-          <t>2. ระยะปีกพับ (Bending Flange): ควรมีความกว้างอย่างน้อย 20 - 30 มม. เพื่อให้จับยึดรีเวทหรือสกรูได้แข็งแรง</t>
+      <c r="A12" s="37" t="inlineStr">
+        <is>
+          <t>4 x 8 ฟุต (ขนาดเต็มแผ่นมาตรฐาน)</t>
+        </is>
+      </c>
+      <c r="B12" s="64" t="n">
+        <v>1220</v>
+      </c>
+      <c r="C12" s="64" t="n">
+        <v>2440</v>
+      </c>
+      <c r="D12" s="32">
+        <f>B12*C12/1000000</f>
+        <v/>
+      </c>
+      <c r="E12" s="26" t="inlineStr">
+        <is>
+          <t>2, 3, 5, 8 มม.</t>
+        </is>
+      </c>
+      <c r="F12" s="26" t="inlineStr">
+        <is>
+          <t>งานตู้โชว์, บานหน้าต่าง, ฝาครอบใส</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="57" t="inlineStr">
-        <is>
-          <t>3. การหาขนาด Blank Size (กว้าง x ยาว ก่อนพับ):</t>
+      <c r="A13" s="37" t="inlineStr">
+        <is>
+          <t>4 x 6 ฟุต (ขนาดตัดแบ่ง)</t>
+        </is>
+      </c>
+      <c r="B13" s="64" t="n">
+        <v>1220</v>
+      </c>
+      <c r="C13" s="64" t="n">
+        <v>1830</v>
+      </c>
+      <c r="D13" s="32">
+        <f>B13*C13/1000000</f>
+        <v/>
+      </c>
+      <c r="E13" s="26" t="inlineStr">
+        <is>
+          <t>2, 3, 5 มม.</t>
+        </is>
+      </c>
+      <c r="F13" s="26" t="inlineStr">
+        <is>
+          <t>ป้ายหน้าร้าน, ฝาครอบเครื่อง</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="57" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   - หากพับขึ้นขอบ 2 ข้าง ซ้าย-ขวา ข้างละ F มม. และแผ่นตรงกลางกว้าง W มม. -&gt; กว้างคลี่ = W + (2 x F) - K-factor (ปกติเผื่อลดลงประมาณ 1-2 มม. ต่อมุมพับ)</t>
+      <c r="A14" s="37" t="inlineStr">
+        <is>
+          <t>3 x 6 ฟุต (ขนาดยอดนิยม)</t>
+        </is>
+      </c>
+      <c r="B14" s="64" t="n">
+        <v>915</v>
+      </c>
+      <c r="C14" s="64" t="n">
+        <v>1830</v>
+      </c>
+      <c r="D14" s="32">
+        <f>B14*C14/1000000</f>
+        <v/>
+      </c>
+      <c r="E14" s="26" t="inlineStr">
+        <is>
+          <t>2, 3, 5 มม.</t>
+        </is>
+      </c>
+      <c r="F14" s="26" t="inlineStr">
+        <is>
+          <t>ชิ้นงานขนาดกลาง ประหยัดเศษ</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="57" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   - เพื่อความปลอดภัยในการสั่งแผ่น สามารถใช้ขนาด กว้างรวมปีก (W + 2F) ได้เลยโดยถือเป็นระยะเผื่อตัดแต่งขอบ</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="57" t="inlineStr">
-        <is>
-          <t>4. ชิ้นงานที่มีชื่อ Arcylic (อะคริลิก): เช่น Arcylic Cover Front, Arcylic Cover Right ให้ตรวจสอบว่าใช้แผ่นอะคริลิกใส หรือแผ่นคอมโพสิตทึบในการตัด</t>
+      <c r="A15" s="37" t="inlineStr">
+        <is>
+          <t>2 x 4 ฟุต (แผ่นเล็ก)</t>
+        </is>
+      </c>
+      <c r="B15" s="64" t="n">
+        <v>610</v>
+      </c>
+      <c r="C15" s="64" t="n">
+        <v>1220</v>
+      </c>
+      <c r="D15" s="32">
+        <f>B15*C15/1000000</f>
+        <v/>
+      </c>
+      <c r="E15" s="26" t="inlineStr">
+        <is>
+          <t>2, 3, 5 มม.</t>
+        </is>
+      </c>
+      <c r="F15" s="26" t="inlineStr">
+        <is>
+          <t>ชิ้นงานขนาดเล็ก, ป้ายไฟ</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="63" t="inlineStr">
+        <is>
+          <t>📐 เทคนิคและข้อแนะนำการตัดและการพับ (Fabrication Notes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="65" t="inlineStr">
+        <is>
+          <t>1. แผ่นคอมโพสิต: ใช้ใบมีดเซาะร่อง V-Groove 90° หรือ 135° ด้านหลัง โดยเหลือชั้นพลาสติกและผิวหน้าไว้ประมาณ 0.5 - 0.8 มม. ก่อนพับขึ้นรูป</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="65" t="inlineStr">
+        <is>
+          <t>2. แผ่นอะคริลิก (Arcylic): แนะนำให้ตัดด้วยเครื่อง Laser Cutting เพื่อให้ขอบเรียบเงาใส ไม่ต้องขัดแต่งเพิ่มเติม</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="65" t="inlineStr">
+        <is>
+          <t>3. ระยะเผื่อคลี่ชิ้นงานพับ (Blank Size): สามารถใช้สูตร กว้างรวมปีกพับ (W + 2F) ในการคำนวณเบื้องต้น เพื่อความปลอดภัยของเศษตัด</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="65" t="inlineStr">
+        <is>
+          <t>4. ค่าเผื่อเศษตัด (Waste Factor): สำหรับอะคริลิกแผ่นใส แนะนำตั้งเผื่อไว้ 15% - 20% เนื่องจากต้องเผื่อระยะแนวทางเดินลำแสงเลเซอร์และการเว้นขอบฟิล์มกันรอย</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="8">
-    <mergeCell ref="A16:F16"/>
-    <mergeCell ref="A11:F11"/>
     <mergeCell ref="A10:F10"/>
-    <mergeCell ref="A13:F13"/>
-    <mergeCell ref="A14:F14"/>
+    <mergeCell ref="A19:F19"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A12:F12"/>
-    <mergeCell ref="A15:F15"/>
+    <mergeCell ref="A17:F17"/>
+    <mergeCell ref="A18:F18"/>
+    <mergeCell ref="A3:F3"/>
+    <mergeCell ref="A21:F21"/>
+    <mergeCell ref="A20:F20"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>